<commit_message>
Added single forms for both trade and position
</commit_message>
<xml_diff>
--- a/src/assets/files/Position-template.xlsx
+++ b/src/assets/files/Position-template.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ensueno Technologies\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DIVYA\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC997CCB-19E5-4A1A-BE30-0976213D4ACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8E4A148-1D27-4B03-9C5F-C96DD9787257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3750" yWindow="1260" windowWidth="24210" windowHeight="14145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="40">
   <si>
     <t>SellAvg</t>
   </si>
@@ -98,6 +98,48 @@
   </si>
   <si>
     <t>NIFTY24080824200PE</t>
+  </si>
+  <si>
+    <t>exchange</t>
+  </si>
+  <si>
+    <t>Instrument type</t>
+  </si>
+  <si>
+    <t>NSE</t>
+  </si>
+  <si>
+    <t>BSE</t>
+  </si>
+  <si>
+    <t>index option2</t>
+  </si>
+  <si>
+    <t>index option8</t>
+  </si>
+  <si>
+    <t>index option4</t>
+  </si>
+  <si>
+    <t>index option3</t>
+  </si>
+  <si>
+    <t>index option5</t>
+  </si>
+  <si>
+    <t>index option6</t>
+  </si>
+  <si>
+    <t>index option7</t>
+  </si>
+  <si>
+    <t>index option9</t>
+  </si>
+  <si>
+    <t>index option10</t>
+  </si>
+  <si>
+    <t>index option11</t>
   </si>
 </sst>
 </file>
@@ -108,10 +150,16 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -475,14 +523,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="10" max="10" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -525,8 +574,14 @@
       <c r="N1" t="s">
         <v>13</v>
       </c>
+      <c r="O1" t="s">
+        <v>26</v>
+      </c>
+      <c r="P1" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>30.8</v>
       </c>
@@ -569,8 +624,14 @@
       <c r="N2">
         <v>12300</v>
       </c>
+      <c r="O2" t="s">
+        <v>28</v>
+      </c>
+      <c r="P2" t="s">
+        <v>30</v>
+      </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>38.85</v>
       </c>
@@ -613,8 +674,14 @@
       <c r="N3">
         <v>12300</v>
       </c>
+      <c r="O3" t="s">
+        <v>29</v>
+      </c>
+      <c r="P3" t="s">
+        <v>33</v>
+      </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>82.4</v>
       </c>
@@ -657,8 +724,14 @@
       <c r="N4">
         <v>12300</v>
       </c>
+      <c r="O4" t="s">
+        <v>28</v>
+      </c>
+      <c r="P4" t="s">
+        <v>32</v>
+      </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>267.39999999999998</v>
       </c>
@@ -701,8 +774,14 @@
       <c r="N5">
         <v>24000</v>
       </c>
+      <c r="O5" t="s">
+        <v>28</v>
+      </c>
+      <c r="P5" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>514.04999999999995</v>
       </c>
@@ -745,8 +824,14 @@
       <c r="N6">
         <v>24000</v>
       </c>
+      <c r="O6" t="s">
+        <v>28</v>
+      </c>
+      <c r="P6" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>67.3125</v>
       </c>
@@ -789,8 +874,14 @@
       <c r="N7">
         <v>12350</v>
       </c>
+      <c r="O7" t="s">
+        <v>28</v>
+      </c>
+      <c r="P7" t="s">
+        <v>36</v>
+      </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>866</v>
       </c>
@@ -824,11 +915,23 @@
       <c r="K8">
         <v>0</v>
       </c>
+      <c r="L8" s="1">
+        <v>45512</v>
+      </c>
       <c r="M8" t="s">
         <v>16</v>
       </c>
+      <c r="N8">
+        <v>785678</v>
+      </c>
+      <c r="O8" t="s">
+        <v>28</v>
+      </c>
+      <c r="P8" t="s">
+        <v>31</v>
+      </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>156.15</v>
       </c>
@@ -871,8 +974,14 @@
       <c r="N9">
         <v>24000</v>
       </c>
+      <c r="O9" t="s">
+        <v>28</v>
+      </c>
+      <c r="P9" t="s">
+        <v>37</v>
+      </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>141.55000000000001</v>
       </c>
@@ -906,11 +1015,23 @@
       <c r="K10">
         <v>0</v>
       </c>
+      <c r="L10" s="1">
+        <v>45512</v>
+      </c>
       <c r="M10" t="s">
         <v>16</v>
       </c>
+      <c r="N10">
+        <v>234</v>
+      </c>
+      <c r="O10" t="s">
+        <v>28</v>
+      </c>
+      <c r="P10" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>246.2</v>
       </c>
@@ -953,8 +1074,15 @@
       <c r="N11">
         <v>24000</v>
       </c>
+      <c r="O11" t="s">
+        <v>28</v>
+      </c>
+      <c r="P11" t="s">
+        <v>39</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>